<commit_message>
Mock 5: round 2 marks of the second review in Cowork (M5-S33 and M5-S45 good). The owner did not mark. The assistant typed the marks on the instruction of the owner.
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TnghEw2ou31QVRW6aTsXeq
</commit_message>
<xml_diff>
--- a/marking/M5-round2.xlsx
+++ b/marking/M5-round2.xlsx
@@ -596,7 +596,11 @@
 D: The guide says that allowed-tools restricts tool access during skill execution, so it does not ask developers for a missing module parameter.</t>
         </is>
       </c>
-      <c r="N2" s="4" t="n"/>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O2" s="4" t="n"/>
     </row>
     <row r="3">
@@ -664,7 +668,11 @@
 D: The guide names the -p flag as the way to run Claude Code in CI. Non-interactive mode does not cause the mix of sure and doubtful findings in one routing decision.</t>
         </is>
       </c>
-      <c r="N3" s="4" t="n"/>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O3" s="4" t="n"/>
     </row>
   </sheetData>

</xml_diff>